<commit_message>
Création du protocol Ships_Astar avec déplacement entre point A et point B simple
</commit_message>
<xml_diff>
--- a/docs/20260911-MIAGE_Astar/20260511-ChronoStageTutoré_2026.1b.xlsx
+++ b/docs/20260911-MIAGE_Astar/20260511-ChronoStageTutoré_2026.1b.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lefur\Documents\GitHub\MelaneSim_2024\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dan\Desktop\Projets\MelaneSim_2024\docs\20260911-MIAGE_Astar\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E45C6193-EAB4-46D0-B235-BC305FBF1071}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AE70718-B9B1-4CA4-9C76-42BD20B6CF08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{8CD262DD-37D0-4D54-B340-C5BBE90D80FB}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8CD262DD-37D0-4D54-B340-C5BBE90D80FB}"/>
   </bookViews>
   <sheets>
     <sheet name="stage 2026.2" sheetId="2" r:id="rId1"/>
@@ -30,15 +30,12 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="64">
   <si>
     <t>Date</t>
   </si>
@@ -221,6 +218,27 @@
   </si>
   <si>
     <t>voir document et humanWalker (protocole Dodel2)</t>
+  </si>
+  <si>
+    <t>création du protocol C_Ships_ASTAR</t>
+  </si>
+  <si>
+    <t>Limitation du nombre de cargos pour garder la scène lisible avec le bateau Astar.</t>
+  </si>
+  <si>
+    <t>Coordonnées de Nouméa et Lifou calculées et vérifiées comme cellules maritimes valides.</t>
+  </si>
+  <si>
+    <t>Création du bateau C_Ship_astar, se déplace en ligne droite de Nouméa à Lifou.</t>
+  </si>
+  <si>
+    <t>Création du protocole Ships_Astar (basé sur Ships), enregistré partout où il fallait (constantes, contexte, IHM, config Repast).</t>
+  </si>
+  <si>
+    <t>Déplacement en ligne droite entre 2 points grâce au nouveau protocol</t>
+  </si>
+  <si>
+    <t>Algorithme Astar pas encore implémenté</t>
   </si>
 </sst>
 </file>
@@ -328,9 +346,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -368,7 +386,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -474,7 +492,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -616,7 +634,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -625,16 +643,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BDC5CEA-2690-4ECE-917D-F43C72E40A35}">
   <dimension ref="A1:D33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.3828125" defaultRowHeight="18.45" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.69140625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="43.69140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="96.3046875" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="102.15234375" style="1" customWidth="1"/>
-    <col min="5" max="16384" width="11.3828125" style="1"/>
+    <col min="1" max="1" width="17.7109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="43.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="143.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="102.140625" style="1" customWidth="1"/>
+    <col min="5" max="16384" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="23.15" x14ac:dyDescent="0.6">
+    <row r="1" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -648,7 +666,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.5">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>46276</v>
       </c>
@@ -659,7 +677,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
       <c r="B3" s="1" t="s">
         <v>49</v>
@@ -668,7 +686,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.5">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="2"/>
       <c r="B4" s="1" t="s">
         <v>50</v>
@@ -677,7 +695,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.5">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="2"/>
       <c r="B5" s="1" t="s">
         <v>51</v>
@@ -686,7 +704,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.5">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="2"/>
       <c r="B6" s="1" t="s">
         <v>52</v>
@@ -695,22 +713,49 @@
         <v>56</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.5">
-      <c r="A7" s="2"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.5">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="2">
+        <v>46291</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="2"/>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="C8" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C9" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C10" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="2"/>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.5">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="2"/>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.5">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A30" s="2"/>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.5">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" s="2"/>
     </row>
   </sheetData>
@@ -722,23 +767,23 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50A5B30A-9091-4023-BC8F-85B7675FB373}">
   <dimension ref="A1:K33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.3828125" defaultRowHeight="18.45" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.69140625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="43.69140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="96.3046875" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="102.15234375" style="1" customWidth="1"/>
-    <col min="5" max="5" width="12.69140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="2.84375" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.69140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.84375" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="2.53515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.3828125" style="1"/>
-    <col min="11" max="11" width="35.53515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="16384" width="11.3828125" style="1"/>
+    <col min="1" max="1" width="17.7109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="43.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="96.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="102.140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="2.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="2.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.42578125" style="1"/>
+    <col min="11" max="11" width="35.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="16384" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="23.15" x14ac:dyDescent="0.6">
+    <row r="1" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -752,7 +797,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>46108</v>
       </c>
@@ -763,7 +808,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>46119</v>
       </c>
@@ -774,7 +819,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>46119</v>
       </c>
@@ -785,7 +830,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>46121</v>
       </c>
@@ -796,7 +841,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>46121</v>
       </c>
@@ -807,7 +852,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>46129</v>
       </c>
@@ -818,7 +863,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>46135</v>
       </c>
@@ -829,32 +874,32 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C9" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C10" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C11" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C12" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C13" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" s="2">
         <v>46023</v>
       </c>
@@ -862,7 +907,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" s="2">
         <v>46146</v>
       </c>
@@ -873,7 +918,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C16" s="1" t="s">
         <v>25</v>
       </c>
@@ -881,13 +926,13 @@
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C17" s="1" t="s">
         <v>43</v>
       </c>
       <c r="K17" s="6"/>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C18" s="1" t="s">
         <v>26</v>
       </c>
@@ -912,7 +957,7 @@
         <v>colorMap.put(1, new Color(21,124,176));</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="E19" t="s">
         <v>30</v>
       </c>
@@ -934,7 +979,7 @@
         <v>colorMap.put(2, new Color(62,146,146));</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="E20" t="s">
         <v>30</v>
       </c>
@@ -956,7 +1001,7 @@
         <v>colorMap.put(3, new Color(104,171,113));</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="E21" t="s">
         <v>30</v>
       </c>
@@ -978,7 +1023,7 @@
         <v>colorMap.put(4, new Color(146,194,82));</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="E22" t="s">
         <v>30</v>
       </c>
@@ -1000,7 +1045,7 @@
         <v>colorMap.put(5, new Color(190,218,49));</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="E23" t="s">
         <v>30</v>
       </c>
@@ -1022,7 +1067,7 @@
         <v>colorMap.put(6, new Color(234,243,16));</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="E24" t="s">
         <v>30</v>
       </c>
@@ -1044,7 +1089,7 @@
         <v>colorMap.put(7, new Color(255,235,0));</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="E25" t="s">
         <v>30</v>
       </c>
@@ -1066,7 +1111,7 @@
         <v>colorMap.put(8, new Color(255,191,0));</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="E26" t="s">
         <v>30</v>
       </c>
@@ -1088,7 +1133,7 @@
         <v>colorMap.put(9, new Color(255,150,0));</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="E27" t="s">
         <v>30</v>
       </c>
@@ -1110,7 +1155,7 @@
         <v>colorMap.put(10, new Color(255,103,0));</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="E28" t="s">
         <v>30</v>
       </c>
@@ -1132,7 +1177,7 @@
         <v>colorMap.put(11, new Color(255,66,0));</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="E29" t="s">
         <v>30</v>
       </c>
@@ -1154,7 +1199,7 @@
         <v>colorMap.put(12, new Color(255,19,0));</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30" s="2">
         <v>46149</v>
       </c>
@@ -1165,17 +1210,17 @@
         <v>45</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C31" s="1" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C32" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.5">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" s="2">
         <v>46153</v>
       </c>

</xml_diff>